<commit_message>
Regenerate BOM with verified SKUs (13 line items, ExaCS X11M + ADB-S + networking)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/output-demo-pharma-mx/opt13-bom.xlsx
+++ b/examples/output-demo-pharma-mx/opt13-bom.xlsx
@@ -90,7 +90,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +107,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8F0F2"/>
         <bgColor rgb="00E8F0F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F4F2"/>
+        <bgColor rgb="00F5F4F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -148,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -183,10 +189,34 @@
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -558,7 +588,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -584,7 +614,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>as of 2026-04-12</t>
+          <t>as of 2026-04-13</t>
         </is>
       </c>
     </row>
@@ -716,85 +746,773 @@
         <v/>
       </c>
       <c r="K7" s="15">
-        <f>IF(J9=0,0,J7/J9)</f>
+        <f>IF(J29=0,0,J7/J29)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>B91961</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>OCI - Block Volume Storage</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>Gigabyte Storage Capacity Per Month</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>0.0255</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="22">
+        <f>D8*E8*F8</f>
+        <v/>
+      </c>
+      <c r="J8" s="22">
+        <f>I8*(1-H8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="23">
+        <f>IF(J29=0,0,J8/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="n"/>
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Subtotal — Oracle Cloud Infrastructure - Storage</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="16" t="n"/>
-      <c r="E8" s="16" t="n"/>
-      <c r="F8" s="16" t="n"/>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="17">
-        <f>SUM(I7:I7)</f>
-        <v/>
-      </c>
-      <c r="J8" s="17">
-        <f>SUM(J7:J7)</f>
-        <v/>
-      </c>
-      <c r="K8" s="16" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="n"/>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="24" t="n"/>
+      <c r="H9" s="24" t="n"/>
+      <c r="I9" s="25">
+        <f>SUM(I7:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="25">
+        <f>SUM(J7:J8)</f>
+        <v/>
+      </c>
+      <c r="K9" s="24" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure - Autonomous Database &amp; Exadata</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>B95703</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Oracle Autonomous Database (ATP or ADW) - BYOL ECPU (2 ECPU minimum)</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>ECPU Per Hour</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>0.08069999999999999</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>744</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="14">
+        <f>D11*E11*F11</f>
+        <v/>
+      </c>
+      <c r="J11" s="14">
+        <f>I11*(1-H11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="15">
+        <f>IF(J29=0,0,J11/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>B95706</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Oracle Autonomous Database Storage for Transaction Processing (ATP), using ECPU</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Gigabyte Storage Capacity Per Month</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>0.1156</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="20" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="22">
+        <f>D12*E12*F12</f>
+        <v/>
+      </c>
+      <c r="J12" s="22">
+        <f>I12*(1-H12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="23">
+        <f>IF(J29=0,0,J12/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="n"/>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Subtotal — Oracle Cloud Infrastructure - Autonomous Database &amp; Exadata</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="24" t="n"/>
+      <c r="F13" s="24" t="n"/>
+      <c r="G13" s="24" t="n"/>
+      <c r="H13" s="24" t="n"/>
+      <c r="I13" s="25">
+        <f>SUM(I11:I12)</f>
+        <v/>
+      </c>
+      <c r="J13" s="25">
+        <f>SUM(J11:J12)</f>
+        <v/>
+      </c>
+      <c r="K13" s="24" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure - Database Exadata Infrastructure</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>B110627</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Cloud Infrastructure - Database Server - X11M</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Hosted Environment Per Hour</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>2.9032</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>744</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="14">
+        <f>D15*E15*F15</f>
+        <v/>
+      </c>
+      <c r="J15" s="14">
+        <f>I15*(1-H15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="15">
+        <f>IF(J29=0,0,J15/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>B110629</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Cloud Infrastructure - Storage Server - X11M</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Hosted Environment Per Hour</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>2.9032</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>744</v>
+      </c>
+      <c r="F16" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="22">
+        <f>D16*E16*F16</f>
+        <v/>
+      </c>
+      <c r="J16" s="22">
+        <f>I16*(1-H16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="23">
+        <f>IF(J29=0,0,J16/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>B110632</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Database ECPU - Dedicated Infrastructure - BYOL (X11M)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>ECPU Per Hour</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>0.08069999999999999</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>744</v>
+      </c>
+      <c r="F17" s="12" t="n">
+        <v>128</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="14">
+        <f>D17*E17*F17</f>
+        <v/>
+      </c>
+      <c r="J17" s="14">
+        <f>I17*(1-H17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="15">
+        <f>IF(J29=0,0,J17/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>B110627</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Cloud Infrastructure - Database Server - X11M</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Hosted Environment Per Hour</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>2.9032</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>744</v>
+      </c>
+      <c r="F18" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="22">
+        <f>D18*E18*F18</f>
+        <v/>
+      </c>
+      <c r="J18" s="22">
+        <f>I18*(1-H18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="23">
+        <f>IF(J29=0,0,J18/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>B110629</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Cloud Infrastructure - Storage Server - X11M</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Hosted Environment Per Hour</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>2.9032</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>744</v>
+      </c>
+      <c r="F19" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="14">
+        <f>D19*E19*F19</f>
+        <v/>
+      </c>
+      <c r="J19" s="14">
+        <f>I19*(1-H19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="15">
+        <f>IF(J29=0,0,J19/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>B110632</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>OCI - Exadata Database ECPU - Dedicated Infrastructure - BYOL (X11M)</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>ECPU Per Hour</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="n">
+        <v>0.08069999999999999</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>744</v>
+      </c>
+      <c r="F20" s="20" t="n">
+        <v>128</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="22">
+        <f>D20*E20*F20</f>
+        <v/>
+      </c>
+      <c r="J20" s="22">
+        <f>I20*(1-H20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="23">
+        <f>IF(J29=0,0,J20/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="n"/>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Subtotal — Oracle Cloud Infrastructure - Database Exadata Infrastructure</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24" t="n"/>
+      <c r="F21" s="24" t="n"/>
+      <c r="G21" s="24" t="n"/>
+      <c r="H21" s="24" t="n"/>
+      <c r="I21" s="25">
+        <f>SUM(I15:I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="25">
+        <f>SUM(J15:J20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="24" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure - Networking</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>B88326</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>OCI - FastConnect 10 Gbps</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Port Hour</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>744</v>
+      </c>
+      <c r="F23" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="H23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="14">
+        <f>D23*E23*F23</f>
+        <v/>
+      </c>
+      <c r="J23" s="14">
+        <f>I23*(1-H23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="15">
+        <f>IF(J29=0,0,J23/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>B88326</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>OCI - FastConnect 10 Gbps</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Port Hour</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>744</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H24" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="22">
+        <f>D24*E24*F24</f>
+        <v/>
+      </c>
+      <c r="J24" s="22">
+        <f>I24*(1-H24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="23">
+        <f>IF(J29=0,0,J24/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="n"/>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Subtotal — Oracle Cloud Infrastructure - Networking</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="24" t="n"/>
+      <c r="G25" s="24" t="n"/>
+      <c r="H25" s="24" t="n"/>
+      <c r="I25" s="25">
+        <f>SUM(I23:I24)</f>
+        <v/>
+      </c>
+      <c r="J25" s="25">
+        <f>SUM(J23:J24)</f>
+        <v/>
+      </c>
+      <c r="K25" s="24" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Oracle Cloud Infrastructure - Security</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>B92092</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>OCI - KMS Vault - Key Versions (Free Tier: 20 Key Versions)</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Key Version Per Month</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>0.5334</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G27" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="H27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="14">
+        <f>D27*E27*F27</f>
+        <v/>
+      </c>
+      <c r="J27" s="14">
+        <f>I27*(1-H27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="15">
+        <f>IF(J29=0,0,J27/J29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="n"/>
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>Subtotal — Oracle Cloud Infrastructure - Security</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
+      <c r="F28" s="24" t="n"/>
+      <c r="G28" s="24" t="n"/>
+      <c r="H28" s="24" t="n"/>
+      <c r="I28" s="25">
+        <f>SUM(I27:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="25">
+        <f>SUM(J27:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="24" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="26" t="n"/>
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="19">
-        <f>I8</f>
-        <v/>
-      </c>
-      <c r="J9" s="19">
-        <f>J8</f>
-        <v/>
-      </c>
-      <c r="K9" s="18" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="C29" s="26" t="n"/>
+      <c r="D29" s="26" t="n"/>
+      <c r="E29" s="26" t="n"/>
+      <c r="F29" s="26" t="n"/>
+      <c r="G29" s="26" t="n"/>
+      <c r="H29" s="26" t="n"/>
+      <c r="I29" s="27">
+        <f>I9+I13+I21+I25+I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="27">
+        <f>J9+J13+J21+J25+J28</f>
+        <v/>
+      </c>
+      <c r="K29" s="26" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="28" t="n"/>
+      <c r="B30" s="29" t="inlineStr">
         <is>
           <t>Annual Run Rate (ARR)</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="20" t="n"/>
-      <c r="F10" s="20" t="n"/>
-      <c r="G10" s="20" t="n"/>
-      <c r="H10" s="20" t="n"/>
-      <c r="I10" s="20" t="n"/>
-      <c r="J10" s="22">
-        <f>J9*12</f>
-        <v/>
-      </c>
-      <c r="K10" s="20" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="C30" s="28" t="n"/>
+      <c r="D30" s="28" t="n"/>
+      <c r="E30" s="28" t="n"/>
+      <c r="F30" s="28" t="n"/>
+      <c r="G30" s="28" t="n"/>
+      <c r="H30" s="28" t="n"/>
+      <c r="I30" s="28" t="n"/>
+      <c r="J30" s="30">
+        <f>J29*12</f>
+        <v/>
+      </c>
+      <c r="K30" s="28" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="31" t="inlineStr">
         <is>
           <t>Disclaimer:</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="24" t="inlineStr">
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t>This sample quote is provided solely for evaluation purposes and is intended to further discussions between you and Oracle. This sample quote is not eligible for acceptance by you and is not a binding contract between you and Oracle for the services specified. If you would like to purchase the services specified in this sample quote, please request that Oracle issue you a formal quote (which may include an OMA or a CSA if you do not already have an appropriate agreement in place with Oracle) for your acceptance and execution. Your formal quote will be effective only upon Oracle's acceptance of the formal quote (and the OMA or CSA, if required).</t>
         </is>
@@ -802,8 +1520,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A33:K33"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A13:K13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add opt13-bom.xlsx with 45% global discount applied
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/output-demo-pharma-mx/opt13-bom.xlsx
+++ b/examples/output-demo-pharma-mx/opt13-bom.xlsx
@@ -735,7 +735,7 @@
         <v>12</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I7" s="14">
         <f>D7*E7*F7</f>
@@ -779,7 +779,7 @@
         <v>12</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I8" s="22">
         <f>D8*E8*F8</f>
@@ -863,7 +863,7 @@
         <v>12</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I11" s="14">
         <f>D11*E11*F11</f>
@@ -907,7 +907,7 @@
         <v>12</v>
       </c>
       <c r="H12" s="21" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I12" s="22">
         <f>D12*E12*F12</f>
@@ -991,7 +991,7 @@
         <v>12</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I15" s="14">
         <f>D15*E15*F15</f>
@@ -1035,7 +1035,7 @@
         <v>12</v>
       </c>
       <c r="H16" s="21" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I16" s="22">
         <f>D16*E16*F16</f>
@@ -1079,7 +1079,7 @@
         <v>12</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I17" s="14">
         <f>D17*E17*F17</f>
@@ -1123,7 +1123,7 @@
         <v>12</v>
       </c>
       <c r="H18" s="21" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I18" s="22">
         <f>D18*E18*F18</f>
@@ -1167,7 +1167,7 @@
         <v>12</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I19" s="14">
         <f>D19*E19*F19</f>
@@ -1211,7 +1211,7 @@
         <v>12</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I20" s="22">
         <f>D20*E20*F20</f>
@@ -1295,7 +1295,7 @@
         <v>12</v>
       </c>
       <c r="H23" s="13" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I23" s="14">
         <f>D23*E23*F23</f>
@@ -1339,7 +1339,7 @@
         <v>12</v>
       </c>
       <c r="H24" s="21" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I24" s="22">
         <f>D24*E24*F24</f>
@@ -1423,7 +1423,7 @@
         <v>12</v>
       </c>
       <c r="H27" s="13" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="I27" s="14">
         <f>D27*E27*F27</f>

</xml_diff>